<commit_message>
using Regex to scan code directly which improve production in finding misconfigurations
</commit_message>
<xml_diff>
--- a/Pulumi_ACID_Research_Data_Management_v1.0.xlsx
+++ b/Pulumi_ACID_Research_Data_Management_v1.0.xlsx
@@ -528,7 +528,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -585,7 +585,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -642,7 +642,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -699,7 +699,7 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -756,7 +756,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">

</xml_diff>